<commit_message>
Version final DIAN-Audit - Certificacion digital con QR funcional
</commit_message>
<xml_diff>
--- a/data/Expedientes Fiscalizacion.xlsx
+++ b/data/Expedientes Fiscalizacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhona\Downloads\AuditCompare\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEBF2A2-48D7-4A9E-8735-A9B59CE2C179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7377EA06-821D-4A38-8B29-38F902339D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{368A5DA1-9F2B-4610-8F7E-40C91CBC159E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>ID Mercancía</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Nike</t>
   </si>
   <si>
-    <t>Negro</t>
-  </si>
-  <si>
     <t>6404.11.00.00</t>
   </si>
   <si>
@@ -86,12 +83,6 @@
     <t>M-0002</t>
   </si>
   <si>
-    <t>Camisetas</t>
-  </si>
-  <si>
-    <t>Adidas</t>
-  </si>
-  <si>
     <t>Azul</t>
   </si>
   <si>
@@ -135,6 +126,9 @@
   </si>
   <si>
     <t>Mercancia verificada</t>
+  </si>
+  <si>
+    <t>Rojo</t>
   </si>
 </sst>
 </file>
@@ -576,10 +570,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -593,89 +587,89 @@
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="E2" s="1">
         <v>250</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="I2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="E3" s="1">
         <v>300</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="E4" s="4">
         <v>150</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="J4" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>